<commit_message>
25 octubre 2021 v2
</commit_message>
<xml_diff>
--- a/_downloads/109b9f5d55724f74347a38b45829e0da/Ejemplo distribución triangular.xlsx
+++ b/_downloads/109b9f5d55724f74347a38b45829e0da/Ejemplo distribución triangular.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\ANÁLISIS DE RIESGOS\Archivos de Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9902A52C-208A-463F-BF0A-6897A5F9E3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5781C5-E538-40A5-B18F-45E6E78188EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{104F5D76-1E87-47BA-AC26-E17CBF973BB8}"/>
   </bookViews>
@@ -69,7 +69,7 @@
     <t>Aleatorio</t>
   </si>
   <si>
-    <t>&gt;=SI(B10&lt;=($C$6-$C$5)/($C$7-$C$5);$C$5+RAIZ(B10*($C$6-$C$5)*($C$7-$C$5));$C$7-RAIZ((1-B10)*($C$6-$C$5)*($C$7-$C$5)))</t>
+    <t>&gt;=SI(B10&lt;=($C$6-$C$5)/($C$7-$C$5);$C$5+RAIZ(B10*($C$6-$C$5)*($C$7-$C$5));$C$7-RAIZ((1-B10)*($C$7-$C$6)*($C$7-$C$5)))</t>
   </si>
 </sst>
 </file>
@@ -193,8 +193,8 @@
       <xdr:row>5</xdr:row>
       <xdr:rowOff>6125</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 12">
@@ -512,7 +512,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 12">
@@ -886,19 +886,19 @@
                         <a:rPr lang="es-MX" sz="900" b="0" i="1">
                           <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                         </a:rPr>
+                        <m:t>𝑐</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>−</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
                         <m:t>𝑏</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>−</m:t>
-                      </m:r>
-                      <m:r>
-                        <a:rPr lang="es-MX" sz="900" b="0" i="1">
-                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        </a:rPr>
-                        <m:t>𝑎</m:t>
                       </m:r>
                       <m:r>
                         <a:rPr lang="es-MX" sz="900" b="0" i="1">
@@ -1176,7 +1176,7 @@
                 <a:rPr lang="es-MX" sz="900" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>[1−𝑃(&lt;𝑥)](𝑏−𝑎)(𝑐−𝑎))</a:t>
+                <a:t>[1−𝑃(&lt;𝑥)](𝑐−𝑏)(𝑐−𝑎))</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="es-CO" sz="900"/>
@@ -1600,15 +1600,15 @@
       </c>
       <c r="B10" s="3">
         <f ca="1">RAND()</f>
-        <v>0.31512280964222639</v>
+        <v>0.44349385975895195</v>
       </c>
       <c r="C10" s="3">
-        <f ca="1">IF(B10&lt;=($C$6-$C$5)/($C$7-$C$5),$C$5+SQRT(B10*($C$6-$C$5)*($C$7-$C$5)),$C$7-SQRT((1-B10)*($C$6-$C$5)*($C$7-$C$5)))</f>
-        <v>986.15029284334469</v>
+        <f ca="1">IF(B10&lt;=($C$6-$C$5)/($C$7-$C$5),$C$5+SQRT(B10*($C$6-$C$5)*($C$7-$C$5)),$C$7-SQRT((1-B10)*($C$7-$C$6)*($C$7-$C$5)))</f>
+        <v>1086.3484196031991</v>
       </c>
       <c r="D10" s="5">
         <f ca="1">INT(C10)</f>
-        <v>986</v>
+        <v>1086</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>11</v>
@@ -1620,15 +1620,15 @@
       </c>
       <c r="B11" s="3">
         <f t="shared" ref="B11:B19" ca="1" si="0">RAND()</f>
-        <v>0.84587625722976745</v>
+        <v>0.52912812704629286</v>
       </c>
       <c r="C11" s="3">
-        <f t="shared" ref="C11:C19" ca="1" si="1">IF(B11&lt;=($C$6-$C$5)/($C$7-$C$5),$C$5+SQRT(B11*($C$6-$C$5)*($C$7-$C$5)),$C$7-SQRT((1-B11)*($C$6-$C$5)*($C$7-$C$5)))</f>
-        <v>1660.0105779914993</v>
+        <f t="shared" ref="C11:C19" ca="1" si="1">IF(B11&lt;=($C$6-$C$5)/($C$7-$C$5),$C$5+SQRT(B11*($C$6-$C$5)*($C$7-$C$5)),$C$7-SQRT((1-B11)*($C$7-$C$6)*($C$7-$C$5)))</f>
+        <v>1159.578790468398</v>
       </c>
       <c r="D11" s="5">
         <f t="shared" ref="D11:D19" ca="1" si="2">INT(C11)</f>
-        <v>1660</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.15">
@@ -1637,15 +1637,15 @@
       </c>
       <c r="B12" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.96050028095840689</v>
+        <v>0.8768832941768766</v>
       </c>
       <c r="C12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1827.8814673511454</v>
+        <v>1570.261639209757</v>
       </c>
       <c r="D12" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1827</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
@@ -1654,15 +1654,15 @@
       </c>
       <c r="B13" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.76072643358896075</v>
+        <v>9.370453905864784E-2</v>
       </c>
       <c r="C13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1576.3785005358209</v>
+        <v>765.10074366924334</v>
       </c>
       <c r="D13" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1576</v>
+        <v>765</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
@@ -1671,15 +1671,15 @@
       </c>
       <c r="B14" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44736531251671274</v>
+        <v>0.37047193401303413</v>
       </c>
       <c r="C14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1356.2018828759551</v>
+        <v>1028.2530684481435</v>
       </c>
       <c r="D14" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1356</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
@@ -1688,15 +1688,15 @@
       </c>
       <c r="B15" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9183678846727884</v>
+        <v>0.92707467074691496</v>
       </c>
       <c r="C15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1752.5649853084478</v>
+        <v>1669.2614418008877</v>
       </c>
       <c r="D15" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1752</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
@@ -1705,15 +1705,15 @@
       </c>
       <c r="B16" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.64667135426079558</v>
+        <v>0.29737669341538608</v>
       </c>
       <c r="C16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1485.2219077074051</v>
+        <v>972.26318939923692</v>
       </c>
       <c r="D16" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1485</v>
+        <v>972</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
@@ -1722,15 +1722,15 @@
       </c>
       <c r="B17" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.41834296155110351</v>
+        <v>0.19922008568715788</v>
       </c>
       <c r="C17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1339.5132258427332</v>
+        <v>886.54244820636245</v>
       </c>
       <c r="D17" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1339</v>
+        <v>886</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
@@ -1739,15 +1739,15 @@
       </c>
       <c r="B18" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.98487482459731401</v>
+        <v>0.57190594387026261</v>
       </c>
       <c r="C18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1893.4923404068304</v>
+        <v>1198.6629397097586</v>
       </c>
       <c r="D18" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1893</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
@@ -1756,15 +1756,15 @@
       </c>
       <c r="B19" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>0.55011665120754327</v>
+        <v>0.34328298716407724</v>
       </c>
       <c r="C19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1419.1278009799896</v>
+        <v>1007.4902926147854</v>
       </c>
       <c r="D19" s="5">
         <f t="shared" ca="1" si="2"/>
-        <v>1419</v>
+        <v>1007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>